<commit_message>
Resolve Meridian ClaimLink narrative-vs-calculated rating conflict
The V-001 security questionnaire's Assessor Findings called ClaimLink's
risk "Critical/High" and "Medium-High," terms that don't exist on the
Vendor Inventory's Risk Rating scale and contradicted that column's own
formula output (Medium, for score 84 under the documented Critical
tier + score < 80 = High / 70-84 = Medium logic). Rewrote the findings
to distinguish the static Critical inherent tier from the calculated
Medium risk rating and state the escalation rationale without silently
overriding the formula. Added a resolved-notes section to the README.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01-meridian-health-grc-program/artifacts/vendor_risk_assessment.xlsx
+++ b/01-meridian-health-grc-program/artifacts/vendor_risk_assessment.xlsx
@@ -24,9 +24,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -145,7 +144,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -201,7 +200,10 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -628,7 +630,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="H5" s="19" t="n">
+      <c r="H5" s="20" t="n">
         <v>45964</v>
       </c>
       <c r="I5" s="15" t="n">
@@ -680,7 +682,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H6" s="19" t="n">
+      <c r="H6" s="20" t="n">
         <v>45944</v>
       </c>
       <c r="I6" s="15" t="n">
@@ -732,7 +734,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H7" s="19" t="n">
+      <c r="H7" s="20" t="n">
         <v>45993</v>
       </c>
       <c r="I7" s="15" t="n">
@@ -784,7 +786,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H8" s="19" t="n">
+      <c r="H8" s="20" t="n">
         <v>45918</v>
       </c>
       <c r="I8" s="15" t="n">
@@ -836,7 +838,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H9" s="19" t="n">
+      <c r="H9" s="20" t="n">
         <v>45959</v>
       </c>
       <c r="I9" s="15" t="n">
@@ -888,7 +890,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="H10" s="19" t="n">
+      <c r="H10" s="20" t="n">
         <v>45890</v>
       </c>
       <c r="I10" s="15" t="n">
@@ -940,7 +942,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="H11" s="19" t="n">
+      <c r="H11" s="20" t="n">
         <v>45980</v>
       </c>
       <c r="I11" s="15" t="n">
@@ -1040,7 +1042,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H13" s="19" t="n">
+      <c r="H13" s="20" t="n">
         <v>46034</v>
       </c>
       <c r="I13" s="15" t="n">
@@ -1092,7 +1094,7 @@
           <t>Partial (bridge letter only)</t>
         </is>
       </c>
-      <c r="H14" s="19" t="n">
+      <c r="H14" s="20" t="n">
         <v>46007</v>
       </c>
       <c r="I14" s="15" t="n">
@@ -1144,7 +1146,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H15" s="19" t="n">
+      <c r="H15" s="20" t="n">
         <v>46057</v>
       </c>
       <c r="I15" s="15" t="n">
@@ -1486,7 +1488,7 @@
     <row r="19" ht="15" customHeight="1" s="11">
       <c r="A19" s="17" t="inlineStr">
         <is>
-          <t>• No current SOC 2 Type II report on file (renewal in progress) — drives Critical/High risk rating pending receipt.</t>
+          <t>• No current SOC 2 Type II report on file (renewal in progress). ClaimLink's static Inherent Risk Tier (Vendor Inventory) is Critical, reflecting its standing PHI/system access; this finding does not by itself change the calculated Risk Rating, but is the basis for the escalated monitoring recommended below.</t>
         </is>
       </c>
     </row>
@@ -1507,7 +1509,7 @@
     <row r="22" ht="23.85" customHeight="1" s="11">
       <c r="A22" s="17" t="inlineStr">
         <is>
-          <t>• Overall assessment score: 84/100 (Medium-High). Recommend conditional approval pending SOC 2 Type II delivery within 90 days; tracked as Risk R-003 in the enterprise Risk Register.</t>
+          <t>• Overall assessment score: 84/100. Per the documented Risk Rating Logic (Scoring Methodology tab: Critical tier + score &lt; 80 = High; score 70-84 = Medium), the calculated Risk Rating is Medium — distinct from the Critical inherent tier, which reflects data sensitivity rather than current control performance. Given the Critical inherent tier and the missing SOC 2 Type II, the assessor recommends conditional approval pending SOC 2 Type II delivery within 90 days, tracked as Risk R-003 in the enterprise Risk Register, notwithstanding the Medium calculated rating.</t>
         </is>
       </c>
     </row>

</xml_diff>